<commit_message>
Actualizar vigilancia normativa 2026-09-13 13:03 UTC
</commit_message>
<xml_diff>
--- a/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
+++ b/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1594"/>
+  <dimension ref="A1:E1607"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43454,6 +43454,357 @@
         </is>
       </c>
     </row>
+    <row r="1595">
+      <c r="A1595" t="inlineStr">
+        <is>
+          <t>2026-09-13 13:03</t>
+        </is>
+      </c>
+      <c r="B1595" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1595" t="inlineStr">
+        <is>
+          <t>11 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1595" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 406 DEL 11 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1595" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 406 DEL 11 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1596">
+      <c r="A1596" t="inlineStr">
+        <is>
+          <t>2026-09-13 13:03</t>
+        </is>
+      </c>
+      <c r="B1596" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1596" t="inlineStr">
+        <is>
+          <t>11 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1596" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 405 DEL 11 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1596" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 405 DEL 11 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1597">
+      <c r="A1597" t="inlineStr">
+        <is>
+          <t>2026-09-13 13:03</t>
+        </is>
+      </c>
+      <c r="B1597" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1597" t="inlineStr">
+        <is>
+          <t>11 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1597" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 404 DEL 11 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1597" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 404 DEL 11 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1598">
+      <c r="A1598" t="inlineStr">
+        <is>
+          <t>2026-09-13 13:03</t>
+        </is>
+      </c>
+      <c r="B1598" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1598" t="inlineStr">
+        <is>
+          <t>11 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1598" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 403 DEL 11 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1598" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 403 DEL 11 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1599">
+      <c r="A1599" t="inlineStr">
+        <is>
+          <t>2026-09-13 13:03</t>
+        </is>
+      </c>
+      <c r="B1599" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1599" t="inlineStr">
+        <is>
+          <t>11 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1599" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 401 DEL 11 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1599" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 401 DEL 11 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1600">
+      <c r="A1600" t="inlineStr">
+        <is>
+          <t>2026-09-13 13:03</t>
+        </is>
+      </c>
+      <c r="B1600" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1600" t="inlineStr">
+        <is>
+          <t>11 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1600" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 402 DEL 11 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1600" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 402 DEL 11 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1601">
+      <c r="A1601" t="inlineStr">
+        <is>
+          <t>2026-09-13 13:03</t>
+        </is>
+      </c>
+      <c r="B1601" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1601" t="inlineStr">
+        <is>
+          <t>11 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1601" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 400 DEL 11 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1601" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 400 DEL 11 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1602">
+      <c r="A1602" t="inlineStr">
+        <is>
+          <t>2026-09-13 13:03</t>
+        </is>
+      </c>
+      <c r="B1602" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1602" t="inlineStr">
+        <is>
+          <t>11 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1602" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 399 DEL 11 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1602" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 399 DEL 11 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1603">
+      <c r="A1603" t="inlineStr">
+        <is>
+          <t>2026-09-13 13:03</t>
+        </is>
+      </c>
+      <c r="B1603" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1603" t="inlineStr">
+        <is>
+          <t>11 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1603" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 398 DEL 11 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1603" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 398 DEL 11 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1604">
+      <c r="A1604" t="inlineStr">
+        <is>
+          <t>2026-09-13 13:03</t>
+        </is>
+      </c>
+      <c r="B1604" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1604" t="inlineStr">
+        <is>
+          <t>11 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1604" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 397 DEL 11 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1604" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 397 DEL 11 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1605">
+      <c r="A1605" t="inlineStr">
+        <is>
+          <t>2026-09-13 13:03</t>
+        </is>
+      </c>
+      <c r="B1605" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1605" t="inlineStr">
+        <is>
+          <t>09 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1605" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 390 DEL 09 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1605" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 390 DEL 09 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1606">
+      <c r="A1606" t="inlineStr">
+        <is>
+          <t>2026-09-13 13:03</t>
+        </is>
+      </c>
+      <c r="B1606" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1606" t="inlineStr">
+        <is>
+          <t>09 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1606" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 391 DEL 09 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1606" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 391 DEL 09 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1607">
+      <c r="A1607" t="inlineStr">
+        <is>
+          <t>2026-09-13 13:03</t>
+        </is>
+      </c>
+      <c r="B1607" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1607" t="inlineStr">
+        <is>
+          <t>09 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1607" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 389 DEL 09 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1607" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 389 DEL 09 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizar vigilancia normativa 2026-09-20 13:03 UTC
</commit_message>
<xml_diff>
--- a/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
+++ b/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1607"/>
+  <dimension ref="A1:E1611"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43805,6 +43805,114 @@
         </is>
       </c>
     </row>
+    <row r="1608">
+      <c r="A1608" t="inlineStr">
+        <is>
+          <t>2026-09-20 13:03</t>
+        </is>
+      </c>
+      <c r="B1608" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1608" t="inlineStr">
+        <is>
+          <t>17 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1608" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 421 DEL 17 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1608" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 421 DEL 17 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1609">
+      <c r="A1609" t="inlineStr">
+        <is>
+          <t>2026-09-20 13:03</t>
+        </is>
+      </c>
+      <c r="B1609" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1609" t="inlineStr">
+        <is>
+          <t>11 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1609" t="inlineStr">
+        <is>
+          <t>RESOLUCION 0949 DEL 11 SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1609" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCION 0949 DEL  11 SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1610">
+      <c r="A1610" t="inlineStr">
+        <is>
+          <t>2026-09-20 13:03</t>
+        </is>
+      </c>
+      <c r="B1610" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1610" t="inlineStr">
+        <is>
+          <t>16 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1610" t="inlineStr">
+        <is>
+          <t>RESOLUCION 01021 DEL 16 SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1610" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCION  01021 DEL 16 SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1611">
+      <c r="A1611" t="inlineStr">
+        <is>
+          <t>2026-09-20 13:03</t>
+        </is>
+      </c>
+      <c r="B1611" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1611" t="inlineStr">
+        <is>
+          <t>15 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1611" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 407 DEL 15 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1611" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 407 DEL 15 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizar vigilancia normativa 2026-09-21 13:03 UTC
</commit_message>
<xml_diff>
--- a/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
+++ b/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1611"/>
+  <dimension ref="A1:E1619"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43913,6 +43913,222 @@
         </is>
       </c>
     </row>
+    <row r="1612">
+      <c r="A1612" t="inlineStr">
+        <is>
+          <t>2026-09-21 13:03</t>
+        </is>
+      </c>
+      <c r="B1612" t="inlineStr">
+        <is>
+          <t>Minhacienda - Proyectos de Decreto 2026</t>
+        </is>
+      </c>
+      <c r="C1612" t="inlineStr">
+        <is>
+          <t>10 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1612" t="inlineStr">
+        <is>
+          <t>PD Por el cual se modifica el Decreto 2555 de 2010, en lo relacionado con el régimen de inversión en activos en el exterior de los fondos de pensiones obligatorias.</t>
+        </is>
+      </c>
+      <c r="E1612" t="inlineStr">
+        <is>
+          <t>https://www.minhacienda.gov.co/normativa/proyectos-de-decretos/2026/documents/20119/2873514/7.+PD+Por+el+cual+se+modifica+el+Decreto+2555+de+2010.pdf/7c69545c-e598-2eb2-38c3-0aafc95a44bf?t=1789061677600</t>
+        </is>
+      </c>
+    </row>
+    <row r="1613">
+      <c r="A1613" t="inlineStr">
+        <is>
+          <t>2026-09-21 13:03</t>
+        </is>
+      </c>
+      <c r="B1613" t="inlineStr">
+        <is>
+          <t>Minhacienda - Proyectos de Decreto 2026</t>
+        </is>
+      </c>
+      <c r="C1613" t="inlineStr">
+        <is>
+          <t>01 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1613" t="inlineStr">
+        <is>
+          <t>PD Medidas aduaneras y de comercio exterior transitorias para mitigar el impacto del terremoto</t>
+        </is>
+      </c>
+      <c r="E1613" t="inlineStr">
+        <is>
+          <t>https://www.minhacienda.gov.co/normativa/proyectos-de-decretos/2026/documents/20119/2873514/PD%2BMJ_II_Publicaci%C3%B3n_medidas_aduaneras_transitorias_010926.pdf/e4316d27-14b2-fc44-cb94-0f8d5accbc70?t=1788301751839</t>
+        </is>
+      </c>
+    </row>
+    <row r="1614">
+      <c r="A1614" t="inlineStr">
+        <is>
+          <t>2026-09-21 13:03</t>
+        </is>
+      </c>
+      <c r="B1614" t="inlineStr">
+        <is>
+          <t>Minhacienda - Proyectos de Decreto 2026</t>
+        </is>
+      </c>
+      <c r="C1614" t="inlineStr">
+        <is>
+          <t>11 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D1614" t="inlineStr">
+        <is>
+          <t>PD Medidas aduaneras transitorias para mitigar el impacto del terremoto</t>
+        </is>
+      </c>
+      <c r="E1614" t="inlineStr">
+        <is>
+          <t>https://www.minhacienda.gov.co/normativa/proyectos-de-decretos/2026/documents/20119/2873514/PD%2BMJ_Meddas_aduaneras_terremoto_110826.pdf/8f2eaecf-9089-44d6-0943-ab125a099d5b?t=1786487011230</t>
+        </is>
+      </c>
+    </row>
+    <row r="1615">
+      <c r="A1615" t="inlineStr">
+        <is>
+          <t>2026-09-21 13:03</t>
+        </is>
+      </c>
+      <c r="B1615" t="inlineStr">
+        <is>
+          <t>Minhacienda - Proyectos de Decreto 2026</t>
+        </is>
+      </c>
+      <c r="C1615" t="inlineStr">
+        <is>
+          <t>11 DE AGOSTO DE 2026</t>
+        </is>
+      </c>
+      <c r="D1615" t="inlineStr">
+        <is>
+          <t>PD Aplazamiento calendario tributario en regiones afectadas por el terremoto</t>
+        </is>
+      </c>
+      <c r="E1615" t="inlineStr">
+        <is>
+          <t>https://www.minhacienda.gov.co/normativa/proyectos-de-decretos/2026/documents/20119/2873514/PD%2BMJ_Aplazamiento_calendario_tributario_110826.pdf/b039f8f7-5827-ea27-86bd-3cfdbbf0c793?t=1786486203591</t>
+        </is>
+      </c>
+    </row>
+    <row r="1616">
+      <c r="A1616" t="inlineStr">
+        <is>
+          <t>2026-09-21 13:03</t>
+        </is>
+      </c>
+      <c r="B1616" t="inlineStr">
+        <is>
+          <t>Minhacienda - Proyectos de Decreto 2026</t>
+        </is>
+      </c>
+      <c r="C1616" t="inlineStr">
+        <is>
+          <t>29 DE JULIO DE 2026</t>
+        </is>
+      </c>
+      <c r="D1616" t="inlineStr">
+        <is>
+          <t>P.D. Por el cual se adiciona un parágrafo al artículo 2.2.8.11.3 del Decreto 1833 de 2016 “Por medio del cual se compilan las normas del Sistema General de Pensiones”</t>
+        </is>
+      </c>
+      <c r="E1616" t="inlineStr">
+        <is>
+          <t>https://www.minhacienda.gov.co/normativa/proyectos-de-decretos/2026/documents/20119/2873514/PD+%2B+Memoria+Justificativa+Omisos.pdf/cae05bef-b36a-7a8e-cdaa-5850e33f9843?t=1785291268794</t>
+        </is>
+      </c>
+    </row>
+    <row r="1617">
+      <c r="A1617" t="inlineStr">
+        <is>
+          <t>2026-09-21 13:03</t>
+        </is>
+      </c>
+      <c r="B1617" t="inlineStr">
+        <is>
+          <t>Minhacienda - Proyectos de Decreto 2026</t>
+        </is>
+      </c>
+      <c r="C1617" t="inlineStr">
+        <is>
+          <t>08 DE JULIO DE 2026</t>
+        </is>
+      </c>
+      <c r="D1617" t="inlineStr">
+        <is>
+          <t>P.D. Por el cual se reglamenta el no cobro de la contribución especial del sector eléctrico a la que hacen referencia los parágrafos 2° y 3°del artículo 211 del Estatuto Tributario.</t>
+        </is>
+      </c>
+      <c r="E1617" t="inlineStr">
+        <is>
+          <t>https://www.minhacienda.gov.co/normativa/proyectos-de-decretos/2026/documents/20119/2873514/PD%2BMJ_Contribuci%C3%B3n_energ%C3%ADa_080726.pdf/a88fa479-0086-f3e5-efe0-d138ce0040b9?t=1783560627210</t>
+        </is>
+      </c>
+    </row>
+    <row r="1618">
+      <c r="A1618" t="inlineStr">
+        <is>
+          <t>2026-09-21 13:03</t>
+        </is>
+      </c>
+      <c r="B1618" t="inlineStr">
+        <is>
+          <t>Minhacienda - Proyectos de Decreto 2026</t>
+        </is>
+      </c>
+      <c r="C1618" t="inlineStr">
+        <is>
+          <t>07 DE JULIO DE 2026</t>
+        </is>
+      </c>
+      <c r="D1618" t="inlineStr">
+        <is>
+          <t>P.D. Por el cual se modifica el artículo 2.17.2.5.1.1. de la Sección 1 del Capítulo 5 del Título 2 de la Parte 17 del Libro 2 del Decreto 1068 de 2015, Único Reglamentario del Sector Hacienda y Crédito Público en lo relacionado con el plazo para el registro de los cambios en los titulares, la destinación o en la empresa receptora de la inversión y de las cancelaciones de las inversiones internacionales</t>
+        </is>
+      </c>
+      <c r="E1618" t="inlineStr">
+        <is>
+          <t>https://www.minhacienda.gov.co/normativa/proyectos-de-decretos/2026/documents/20119/2873514/MinComercio_PD_Elmininaci%C3%B3n_t%C3%A9rmino_registro.pdf/93e6d92d-7e5f-1789-f452-c00c60b861a8?t=1783450662988</t>
+        </is>
+      </c>
+    </row>
+    <row r="1619">
+      <c r="A1619" t="inlineStr">
+        <is>
+          <t>2026-09-21 13:03</t>
+        </is>
+      </c>
+      <c r="B1619" t="inlineStr">
+        <is>
+          <t>Minhacienda - Proyectos de Decreto 2026</t>
+        </is>
+      </c>
+      <c r="C1619" t="inlineStr">
+        <is>
+          <t>07 DE JULIO DE 2026</t>
+        </is>
+      </c>
+      <c r="D1619" t="inlineStr">
+        <is>
+          <t>P.D. Por el cual se adiciona el Título 16 a la Parte 11 del Libro 2 al Decreto 1068 de 2015, en lo relacionado con los planes de fortalecimiento institucional, planes de resolución y mecanismos de articulación de resolución para las organizaciones de la economía solidaria que prestan servicios de ahorro y crédito, y se dictan otras disposiciones.</t>
+        </is>
+      </c>
+      <c r="E1619" t="inlineStr">
+        <is>
+          <t>https://www.minhacienda.gov.co/normativa/proyectos-de-decretos/2026/documents/20119/2873514/P.D.++planes%C2%A0de%C2%A0fortalecimiento%C2%A0institucional.pdf/4d6a55d0-dbbc-2efc-8fd5-332dde27b390?t=1783443925392</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizar vigilancia normativa 2026-09-22 13:04 UTC
</commit_message>
<xml_diff>
--- a/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
+++ b/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1619"/>
+  <dimension ref="A1:E1620"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44129,6 +44129,33 @@
         </is>
       </c>
     </row>
+    <row r="1620">
+      <c r="A1620" t="inlineStr">
+        <is>
+          <t>2026-09-22 13:04</t>
+        </is>
+      </c>
+      <c r="B1620" t="inlineStr">
+        <is>
+          <t>Presidencia - Leyes</t>
+        </is>
+      </c>
+      <c r="C1620" t="inlineStr">
+        <is>
+          <t>14 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1620" t="inlineStr">
+        <is>
+          <t>LEY No. 2633 DEL 14 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1620" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/LEY No. 2633 DEL 14 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizar vigilancia normativa 2026-09-23 13:05 UTC
</commit_message>
<xml_diff>
--- a/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
+++ b/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1620"/>
+  <dimension ref="A1:E1621"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44156,6 +44156,33 @@
         </is>
       </c>
     </row>
+    <row r="1621">
+      <c r="A1621" t="inlineStr">
+        <is>
+          <t>2026-09-23 13:05</t>
+        </is>
+      </c>
+      <c r="B1621" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1621" t="inlineStr">
+        <is>
+          <t>21 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1621" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 429 DEL 21 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1621" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 429 DEL 21 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizar vigilancia normativa 2026-10-03 16:51 UTC
</commit_message>
<xml_diff>
--- a/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
+++ b/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1621"/>
+  <dimension ref="A1:E1627"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44183,6 +44183,168 @@
         </is>
       </c>
     </row>
+    <row r="1622">
+      <c r="A1622" t="inlineStr">
+        <is>
+          <t>2026-10-03 16:51</t>
+        </is>
+      </c>
+      <c r="B1622" t="inlineStr">
+        <is>
+          <t>Presidencia - Leyes</t>
+        </is>
+      </c>
+      <c r="C1622" t="inlineStr">
+        <is>
+          <t>1 DE OCTUBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1622" t="inlineStr">
+        <is>
+          <t>LEY No. 2638 DEL 1 DE OCTUBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1622" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/LEY No. 2638 DEL 1 DE OCTUBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1623">
+      <c r="A1623" t="inlineStr">
+        <is>
+          <t>2026-10-03 16:51</t>
+        </is>
+      </c>
+      <c r="B1623" t="inlineStr">
+        <is>
+          <t>Presidencia - Leyes</t>
+        </is>
+      </c>
+      <c r="C1623" t="inlineStr">
+        <is>
+          <t>30 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1623" t="inlineStr">
+        <is>
+          <t>LEY No. 2637 DEL 30 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1623" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/LEY No. 2637 DEL 30 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1624">
+      <c r="A1624" t="inlineStr">
+        <is>
+          <t>2026-10-03 16:51</t>
+        </is>
+      </c>
+      <c r="B1624" t="inlineStr">
+        <is>
+          <t>Presidencia - Leyes</t>
+        </is>
+      </c>
+      <c r="C1624" t="inlineStr">
+        <is>
+          <t>30 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1624" t="inlineStr">
+        <is>
+          <t>LEY No. 2636 DEL 30 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1624" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/LEY No. 2636 DEL 30 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1625">
+      <c r="A1625" t="inlineStr">
+        <is>
+          <t>2026-10-03 16:51</t>
+        </is>
+      </c>
+      <c r="B1625" t="inlineStr">
+        <is>
+          <t>Presidencia - Leyes</t>
+        </is>
+      </c>
+      <c r="C1625" t="inlineStr">
+        <is>
+          <t>22 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1625" t="inlineStr">
+        <is>
+          <t>LEY No. 2635 DEL 22 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1625" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/LEY No. 2635 DEL 22 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1626">
+      <c r="A1626" t="inlineStr">
+        <is>
+          <t>2026-10-03 16:51</t>
+        </is>
+      </c>
+      <c r="B1626" t="inlineStr">
+        <is>
+          <t>Presidencia - Leyes</t>
+        </is>
+      </c>
+      <c r="C1626" t="inlineStr">
+        <is>
+          <t>22 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1626" t="inlineStr">
+        <is>
+          <t>LEY No. 2634 DEL 22 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1626" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/LEY No. 2634 DEL 22 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1627">
+      <c r="A1627" t="inlineStr">
+        <is>
+          <t>2026-10-03 16:51</t>
+        </is>
+      </c>
+      <c r="B1627" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1627" t="inlineStr">
+        <is>
+          <t>28 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1627" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 431 DEL 28 DE SEPTIEMBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1627" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 431 DEL 28 DE SEPTIEMBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizar vigilancia normativa 2026-10-07 19:10 UTC
</commit_message>
<xml_diff>
--- a/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
+++ b/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1627"/>
+  <dimension ref="A1:E1628"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44345,6 +44345,33 @@
         </is>
       </c>
     </row>
+    <row r="1628">
+      <c r="A1628" t="inlineStr">
+        <is>
+          <t>2026-10-07 19:10</t>
+        </is>
+      </c>
+      <c r="B1628" t="inlineStr">
+        <is>
+          <t>Presidencia - Resoluciones</t>
+        </is>
+      </c>
+      <c r="C1628" t="inlineStr">
+        <is>
+          <t>6 DE OCTUBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1628" t="inlineStr">
+        <is>
+          <t>RESOLUCIÓN EJECUTIVA 455 DEL 6 DE OCTUBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1628" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/RESOLUCIÓN EJECUTIVA 455 DEL 6 DE OCTUBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizar vigilancia normativa 2026-10-18 16:13 UTC
</commit_message>
<xml_diff>
--- a/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
+++ b/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1628"/>
+  <dimension ref="A1:E1629"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44372,6 +44372,33 @@
         </is>
       </c>
     </row>
+    <row r="1629">
+      <c r="A1629" t="inlineStr">
+        <is>
+          <t>2026-10-18 16:13</t>
+        </is>
+      </c>
+      <c r="B1629" t="inlineStr">
+        <is>
+          <t>Presidencia - Circulares</t>
+        </is>
+      </c>
+      <c r="C1629" t="inlineStr">
+        <is>
+          <t>14 DE OCTUBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1629" t="inlineStr">
+        <is>
+          <t>CIRCULAR INTERNA No. 07 DE 2026</t>
+        </is>
+      </c>
+      <c r="E1629" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/CIRCULAR INTERNA No. 07 DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizar vigilancia normativa 2026-10-24 16:20 UTC
</commit_message>
<xml_diff>
--- a/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
+++ b/C:\Users\priesgo\OneDrive - ASOBANCARIA\Documentos\Automatización\VigilanciaNormativa\normativa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1629"/>
+  <dimension ref="A1:E1630"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44399,6 +44399,33 @@
         </is>
       </c>
     </row>
+    <row r="1630">
+      <c r="A1630" t="inlineStr">
+        <is>
+          <t>2026-10-24 16:20</t>
+        </is>
+      </c>
+      <c r="B1630" t="inlineStr">
+        <is>
+          <t>Presidencia - Leyes</t>
+        </is>
+      </c>
+      <c r="C1630" t="inlineStr">
+        <is>
+          <t>20 DE OCTUBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="D1630" t="inlineStr">
+        <is>
+          <t>LEY No. 2639 DEL 20 DE OCTUBRE DE 2026</t>
+        </is>
+      </c>
+      <c r="E1630" t="inlineStr">
+        <is>
+          <t>https://dapre.presidencia.gov.co/normativa/normativa/LEY No. 2639 DEL 20 DE OCTUBRE DE 2026.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>